<commit_message>
Rebuild Growth Pack sample workbook
</commit_message>
<xml_diff>
--- a/portfolio/growth-packs/sample/sample-growth-pack.xlsx
+++ b/portfolio/growth-packs/sample/sample-growth-pack.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="1" r:id="Ra79125ce2cb34950"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="2" r:id="R592e4a258d3b4aaf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="1" r:id="Rfa6192b40fda4dda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="2" r:id="Rb20951a25c7243c9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,21 +14,56 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="9">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
-      <x:sz val="20"/>
+      <x:sz val="16"/>
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF344054"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FF5E5965"/>
+      <x:color rgb="FF17233C"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF243044"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1C6B3A"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF8A6116"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF475467"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
@@ -38,37 +73,13 @@
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FF36523A"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FF6E5A1D"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FF6A625B"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
       <x:i/>
       <x:sz val="11"/>
-      <x:color rgb="FF6A7073"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="18"/>
-      <x:color rgb="FFFFFFFF"/>
+      <x:color rgb="FF344054"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -77,186 +88,288 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF1C252B"/>
+        <x:fgColor rgb="FF17233C"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFEEE9F3"/>
+        <x:fgColor rgb="FFEEF2F6"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF263239"/>
+        <x:fgColor rgb="FFF8FAFC"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFDCE9DD"/>
+        <x:fgColor rgb="FF23395B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFF3EBCF"/>
+        <x:fgColor rgb="FFE8F5EC"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFECE7E1"/>
+        <x:fgColor rgb="FFFFF6D8"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFF8F5EF"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFF4F0E9"/>
+        <x:fgColor rgb="FFF2F4F7"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="8">
     <x:border/>
     <x:border/>
+    <x:border>
+      <x:left/>
+      <x:top/>
+      <x:bottom/>
+    </x:border>
+    <x:border>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:top/>
+      <x:bottom/>
+    </x:border>
+    <x:border>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+    </x:border>
+    <x:border>
+      <x:bottom/>
+    </x:border>
+    <x:border>
+      <x:bottom/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="58">
+  <x:cellXfs count="91">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center"/>
+      <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center"/>
+      <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -266,7 +379,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GrowthPackSample" displayName="GrowthPackSample" ref="A4:J12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SampleProspectsTable" displayName="SampleProspectsTable" ref="A6:J14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Priority"/>
     <x:tableColumn id="2" name="Prospect"/>
@@ -482,31 +595,31 @@
     <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="38" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="42" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="5" t="str">
-        <x:v>BMC Local Growth Pack</x:v>
-      </x:c>
-      <x:c r="B1" s="5"/>
-      <x:c r="C1" s="5"/>
-      <x:c r="D1" s="5"/>
-      <x:c r="E1" s="5"/>
-      <x:c r="F1" s="5"/>
-      <x:c r="G1" s="5"/>
-      <x:c r="H1" s="5"/>
-      <x:c r="I1" s="5"/>
-      <x:c r="J1" s="5"/>
-    </x:row>
-    <x:row r="2" ht="22" customHeight="1">
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>BMC Local Growth Pack — Sample Prospect List</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+      <x:c r="I1" s="4"/>
+      <x:c r="J1" s="4"/>
+    </x:row>
+    <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>Illustrative prospect sample • Commercial cleaning seller • Fictional companies</x:v>
+        <x:v>Illustrative sample for a commercial cleaning seller. Fictional companies and contact details are used so buyers can evaluate the structure of the deliverable.</x:v>
       </x:c>
       <x:c r="B2" s="11"/>
       <x:c r="C2" s="11"/>
@@ -518,317 +631,334 @@
       <x:c r="I2" s="11"/>
       <x:c r="J2" s="11"/>
     </x:row>
-    <x:row r="4" ht="26" customHeight="1">
-      <x:c r="A4" s="16" t="str">
+    <x:row r="4">
+      <x:c r="A4" s="20" t="str">
+        <x:v>Sample rows</x:v>
+      </x:c>
+      <x:c r="B4" s="21" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C4" s="20" t="str">
+        <x:v>Priority A</x:v>
+      </x:c>
+      <x:c r="D4" s="21" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E4" s="20" t="str">
+        <x:v>Priority B</x:v>
+      </x:c>
+      <x:c r="F4" s="21" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G4" s="20" t="str">
+        <x:v>Priority C</x:v>
+      </x:c>
+      <x:c r="H4" s="21" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I4" s="20" t="str">
+        <x:v>Example market</x:v>
+      </x:c>
+      <x:c r="J4" s="21" t="str">
+        <x:v>Northern Arizona</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="32" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="B4" s="16" t="str">
+      <x:c r="B6" s="32" t="str">
         <x:v>Prospect</x:v>
       </x:c>
-      <x:c r="C4" s="16" t="str">
+      <x:c r="C6" s="32" t="str">
         <x:v>Market</x:v>
       </x:c>
-      <x:c r="D4" s="16" t="str">
+      <x:c r="D6" s="32" t="str">
         <x:v>Website</x:v>
       </x:c>
-      <x:c r="E4" s="16" t="str">
+      <x:c r="E6" s="32" t="str">
         <x:v>Public Email</x:v>
       </x:c>
-      <x:c r="F4" s="16" t="str">
+      <x:c r="F6" s="32" t="str">
         <x:v>Public Phone</x:v>
       </x:c>
-      <x:c r="G4" s="16" t="str">
+      <x:c r="G6" s="32" t="str">
         <x:v>Why It Fits</x:v>
       </x:c>
-      <x:c r="H4" s="16" t="str">
+      <x:c r="H6" s="32" t="str">
         <x:v>Likely Need</x:v>
       </x:c>
-      <x:c r="I4" s="16" t="str">
+      <x:c r="I6" s="32" t="str">
         <x:v>Suggested Outreach Angle</x:v>
       </x:c>
-      <x:c r="J4" s="16" t="str">
+      <x:c r="J6" s="32" t="str">
         <x:v>Research Status</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="62" customHeight="1">
-      <x:c r="A5" s="27" t="str">
+    <x:row r="7" ht="54" customHeight="1">
+      <x:c r="A7" s="53" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="B5" s="22" t="str">
+      <x:c r="B7" s="42" t="str">
         <x:v>Juniper Ridge Dental Group</x:v>
       </x:c>
-      <x:c r="C5" s="22" t="str">
+      <x:c r="C7" s="42" t="str">
         <x:v>Prescott, AZ</x:v>
       </x:c>
-      <x:c r="D5" s="22" t="str">
+      <x:c r="D7" s="42" t="str">
         <x:v>https://example.com</x:v>
       </x:c>
-      <x:c r="E5" s="22" t="str">
+      <x:c r="E7" s="42" t="str">
         <x:v>facilities@example.com</x:v>
       </x:c>
-      <x:c r="F5" s="22" t="str">
+      <x:c r="F7" s="42" t="str">
         <x:v>928-555-0101</x:v>
       </x:c>
-      <x:c r="G5" s="22" t="str">
+      <x:c r="G7" s="42" t="str">
         <x:v>Multi-provider dental office with patient-facing space and likely after-hours access needs.</x:v>
       </x:c>
-      <x:c r="H5" s="22" t="str">
+      <x:c r="H7" s="42" t="str">
         <x:v>Recurring evening cleaning</x:v>
       </x:c>
-      <x:c r="I5" s="22" t="str">
+      <x:c r="I7" s="42" t="str">
         <x:v>Keep patient areas ready without adding more vendor coordination.</x:v>
       </x:c>
-      <x:c r="J5" s="22" t="str">
+      <x:c r="J7" s="42" t="str">
         <x:v>Illustrative sample</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="62" customHeight="1">
-      <x:c r="A6" s="27" t="str">
+    <x:row r="8" ht="54" customHeight="1">
+      <x:c r="A8" s="53" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="B6" s="48" t="str">
+      <x:c r="B8" s="42" t="str">
         <x:v>High Desert Property Partners</x:v>
       </x:c>
-      <x:c r="C6" s="48" t="str">
+      <x:c r="C8" s="42" t="str">
         <x:v>Prescott Valley, AZ</x:v>
       </x:c>
-      <x:c r="D6" s="48" t="str">
+      <x:c r="D8" s="42" t="str">
         <x:v>https://example.com</x:v>
       </x:c>
-      <x:c r="E6" s="48" t="str">
+      <x:c r="E8" s="42" t="str">
         <x:v>operations@example.com</x:v>
       </x:c>
-      <x:c r="F6" s="48" t="str">
+      <x:c r="F8" s="42" t="str">
         <x:v>928-555-0102</x:v>
       </x:c>
-      <x:c r="G6" s="48" t="str">
+      <x:c r="G8" s="42" t="str">
         <x:v>Manages multiple small commercial properties with recurring turnovers and common areas.</x:v>
       </x:c>
-      <x:c r="H6" s="48" t="str">
+      <x:c r="H8" s="42" t="str">
         <x:v>Turnover + common-area cleaning</x:v>
       </x:c>
-      <x:c r="I6" s="48" t="str">
+      <x:c r="I8" s="42" t="str">
         <x:v>Use one cleaning relationship across vacancies, turnovers, and shared spaces.</x:v>
       </x:c>
-      <x:c r="J6" s="48" t="str">
+      <x:c r="J8" s="42" t="str">
         <x:v>Illustrative sample</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="62" customHeight="1">
-      <x:c r="A7" s="27" t="str">
+    <x:row r="9" ht="54" customHeight="1">
+      <x:c r="A9" s="53" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="B7" s="22" t="str">
+      <x:c r="B9" s="42" t="str">
         <x:v>Ponderosa Pediatric Clinic</x:v>
       </x:c>
-      <x:c r="C7" s="22" t="str">
+      <x:c r="C9" s="42" t="str">
         <x:v>Prescott Valley, AZ</x:v>
       </x:c>
-      <x:c r="D7" s="22" t="str">
+      <x:c r="D9" s="42" t="str">
         <x:v>https://example.com</x:v>
       </x:c>
-      <x:c r="E7" s="22" t="str">
+      <x:c r="E9" s="42" t="str">
         <x:v>office@example.com</x:v>
       </x:c>
-      <x:c r="F7" s="22" t="str">
+      <x:c r="F9" s="42" t="str">
         <x:v>928-555-0104</x:v>
       </x:c>
-      <x:c r="G7" s="22" t="str">
+      <x:c r="G9" s="42" t="str">
         <x:v>Busy patient-facing medical office where consistent after-hours reset matters.</x:v>
       </x:c>
-      <x:c r="H7" s="22" t="str">
+      <x:c r="H9" s="42" t="str">
         <x:v>Recurring office cleaning</x:v>
       </x:c>
-      <x:c r="I7" s="22" t="str">
+      <x:c r="I9" s="42" t="str">
         <x:v>Reliable after-hours cleaning built around patient traffic and staff schedules.</x:v>
       </x:c>
-      <x:c r="J7" s="22" t="str">
+      <x:c r="J9" s="42" t="str">
         <x:v>Illustrative sample</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="62" customHeight="1">
-      <x:c r="A8" s="35" t="str">
+    <x:row r="10" ht="54" customHeight="1">
+      <x:c r="A10" s="61" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="B8" s="48" t="str">
+      <x:c r="B10" s="42" t="str">
         <x:v>Copper State Fitness Center</x:v>
       </x:c>
-      <x:c r="C8" s="48" t="str">
+      <x:c r="C10" s="42" t="str">
         <x:v>Prescott, AZ</x:v>
       </x:c>
-      <x:c r="D8" s="48" t="str">
+      <x:c r="D10" s="42" t="str">
         <x:v>https://example.com</x:v>
       </x:c>
-      <x:c r="E8" s="48" t="str">
+      <x:c r="E10" s="42" t="str">
         <x:v>manager@example.com</x:v>
       </x:c>
-      <x:c r="F8" s="48" t="str">
+      <x:c r="F10" s="42" t="str">
         <x:v>928-555-0103</x:v>
       </x:c>
-      <x:c r="G8" s="48" t="str">
+      <x:c r="G10" s="42" t="str">
         <x:v>High-touch gym environment with recurring floor, restroom, and sanitation demand.</x:v>
       </x:c>
-      <x:c r="H8" s="48" t="str">
+      <x:c r="H10" s="42" t="str">
         <x:v>Recurring sanitation + floor care</x:v>
       </x:c>
-      <x:c r="I8" s="48" t="str">
+      <x:c r="I10" s="42" t="str">
         <x:v>Build the cleaning schedule around operating hours and heavy-use areas.</x:v>
       </x:c>
-      <x:c r="J8" s="48" t="str">
+      <x:c r="J10" s="42" t="str">
         <x:v>Illustrative sample</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="62" customHeight="1">
-      <x:c r="A9" s="35" t="str">
+    <x:row r="11" ht="54" customHeight="1">
+      <x:c r="A11" s="61" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="B9" s="22" t="str">
+      <x:c r="B11" s="42" t="str">
         <x:v>Granite Peak Business Suites</x:v>
       </x:c>
-      <x:c r="C9" s="22" t="str">
+      <x:c r="C11" s="42" t="str">
         <x:v>Prescott, AZ</x:v>
       </x:c>
-      <x:c r="D9" s="22" t="str">
+      <x:c r="D11" s="42" t="str">
         <x:v>https://example.com</x:v>
       </x:c>
-      <x:c r="E9" s="22" t="str">
+      <x:c r="E11" s="42" t="str">
         <x:v>leasing@example.com</x:v>
       </x:c>
-      <x:c r="F9" s="22" t="str">
+      <x:c r="F11" s="42" t="str">
         <x:v>928-555-0105</x:v>
       </x:c>
-      <x:c r="G9" s="22" t="str">
+      <x:c r="G11" s="42" t="str">
         <x:v>Shared office suites create common-area work plus periodic vacancy cleaning.</x:v>
       </x:c>
-      <x:c r="H9" s="22" t="str">
+      <x:c r="H11" s="42" t="str">
         <x:v>Common-area + vacancy cleaning</x:v>
       </x:c>
-      <x:c r="I9" s="22" t="str">
+      <x:c r="I11" s="42" t="str">
         <x:v>Flexible service that scales with tenant turnover and shared-space needs.</x:v>
       </x:c>
-      <x:c r="J9" s="22" t="str">
+      <x:c r="J11" s="42" t="str">
         <x:v>Illustrative sample</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="62" customHeight="1">
-      <x:c r="A10" s="35" t="str">
+    <x:row r="12" ht="54" customHeight="1">
+      <x:c r="A12" s="61" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="B10" s="48" t="str">
+      <x:c r="B12" s="42" t="str">
         <x:v>Willow Creek Senior Living</x:v>
       </x:c>
-      <x:c r="C10" s="48" t="str">
+      <x:c r="C12" s="42" t="str">
         <x:v>Prescott, AZ</x:v>
       </x:c>
-      <x:c r="D10" s="48" t="str">
+      <x:c r="D12" s="42" t="str">
         <x:v>https://example.com</x:v>
       </x:c>
-      <x:c r="E10" s="48" t="str">
+      <x:c r="E12" s="42" t="str">
         <x:v>admin@example.com</x:v>
       </x:c>
-      <x:c r="F10" s="48" t="str">
+      <x:c r="F12" s="42" t="str">
         <x:v>928-555-0106</x:v>
       </x:c>
-      <x:c r="G10" s="48" t="str">
+      <x:c r="G12" s="42" t="str">
         <x:v>Senior-living environment with recurring common-area needs and high cleanliness expectations.</x:v>
       </x:c>
-      <x:c r="H10" s="48" t="str">
+      <x:c r="H12" s="42" t="str">
         <x:v>Recurring janitorial + floor care</x:v>
       </x:c>
-      <x:c r="I10" s="48" t="str">
+      <x:c r="I12" s="42" t="str">
         <x:v>Consistent scheduled service with extra attention to entrances, halls, and shared areas.</x:v>
       </x:c>
-      <x:c r="J10" s="48" t="str">
+      <x:c r="J12" s="42" t="str">
         <x:v>Illustrative sample</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="62" customHeight="1">
-      <x:c r="A11" s="43" t="str">
+    <x:row r="13" ht="54" customHeight="1">
+      <x:c r="A13" s="69" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="B11" s="22" t="str">
+      <x:c r="B13" s="42" t="str">
         <x:v>Mingus View Business Park</x:v>
       </x:c>
-      <x:c r="C11" s="22" t="str">
+      <x:c r="C13" s="42" t="str">
         <x:v>Cottonwood, AZ</x:v>
       </x:c>
-      <x:c r="D11" s="22" t="str">
+      <x:c r="D13" s="42" t="str">
         <x:v>https://example.com</x:v>
       </x:c>
-      <x:c r="E11" s="22" t="str">
+      <x:c r="E13" s="42" t="str">
         <x:v>property@example.com</x:v>
       </x:c>
-      <x:c r="F11" s="22" t="str">
+      <x:c r="F13" s="42" t="str">
         <x:v>928-555-0107</x:v>
       </x:c>
-      <x:c r="G11" s="22" t="str">
+      <x:c r="G13" s="42" t="str">
         <x:v>Small multi-tenant commercial property with periodic tenant turnover and exterior traffic.</x:v>
       </x:c>
-      <x:c r="H11" s="22" t="str">
+      <x:c r="H13" s="42" t="str">
         <x:v>Common-area + move-out cleaning</x:v>
       </x:c>
-      <x:c r="I11" s="22" t="str">
+      <x:c r="I13" s="42" t="str">
         <x:v>Offer a simple property-wide cleaning option instead of coordinating one-off vendors.</x:v>
       </x:c>
-      <x:c r="J11" s="22" t="str">
+      <x:c r="J13" s="42" t="str">
         <x:v>Illustrative sample</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="62" customHeight="1">
-      <x:c r="A12" s="43" t="str">
+    <x:row r="14" ht="54" customHeight="1">
+      <x:c r="A14" s="77" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="B12" s="48" t="str">
+      <x:c r="B14" s="43" t="str">
         <x:v>Verde Valley Wellness Center</x:v>
       </x:c>
-      <x:c r="C12" s="48" t="str">
+      <x:c r="C14" s="43" t="str">
         <x:v>Cottonwood, AZ</x:v>
       </x:c>
-      <x:c r="D12" s="48" t="str">
+      <x:c r="D14" s="43" t="str">
         <x:v>https://example.com</x:v>
       </x:c>
-      <x:c r="E12" s="48" t="str">
+      <x:c r="E14" s="43" t="str">
         <x:v>office@example.com</x:v>
       </x:c>
-      <x:c r="F12" s="48" t="str">
+      <x:c r="F14" s="43" t="str">
         <x:v>928-555-0108</x:v>
       </x:c>
-      <x:c r="G12" s="48" t="str">
+      <x:c r="G14" s="43" t="str">
         <x:v>Appointment-based wellness office with customer-facing rooms and predictable closing hours.</x:v>
       </x:c>
-      <x:c r="H12" s="48" t="str">
+      <x:c r="H14" s="43" t="str">
         <x:v>Evening office cleaning</x:v>
       </x:c>
-      <x:c r="I12" s="48" t="str">
+      <x:c r="I14" s="43" t="str">
         <x:v>Position around dependable after-hours resets that do not disrupt appointments.</x:v>
       </x:c>
-      <x:c r="J12" s="48" t="str">
+      <x:c r="J14" s="43" t="str">
         <x:v>Illustrative sample</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="51" t="str">
-        <x:v>Sample only. A paid pack is researched for the buyer's actual market, ideal customer, and offer.</x:v>
-      </x:c>
-      <x:c r="B14" s="51"/>
-      <x:c r="C14" s="51"/>
-      <x:c r="D14" s="51"/>
-      <x:c r="E14" s="51"/>
-      <x:c r="F14" s="51"/>
-      <x:c r="G14" s="51"/>
-      <x:c r="H14" s="51"/>
-      <x:c r="I14" s="51"/>
-      <x:c r="J14" s="51"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J1"/>
     <x:mergeCell ref="A2:J2"/>
-    <x:mergeCell ref="A14:J14"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra03d3efd903a42f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69b3335df0a74e63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -837,62 +967,126 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="52" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="54" t="str">
-        <x:v>How to Use the Growth Pack</x:v>
-      </x:c>
-      <x:c r="B1" s="54"/>
-      <x:c r="C1" s="54"/>
-      <x:c r="D1" s="54"/>
+      <x:c r="A1" s="3" t="str">
+        <x:v>What a BMC Local Growth Pack contains</x:v>
+      </x:c>
+      <x:c r="B1" s="3"/>
+      <x:c r="C1" s="3"/>
+      <x:c r="D1" s="3"/>
+      <x:c r="E1" s="3"/>
+      <x:c r="F1" s="3"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="56" t="str">
+      <x:c r="A3" s="82" t="str">
+        <x:v>Field</x:v>
+      </x:c>
+      <x:c r="B3" s="82" t="str">
+        <x:v>What it means</x:v>
+      </x:c>
+      <x:c r="C3" s="82" t="str"/>
+      <x:c r="D3" s="82" t="str"/>
+      <x:c r="E3" s="82" t="str"/>
+      <x:c r="F3" s="82" t="str"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="85" t="str">
+        <x:v>Prospect</x:v>
+      </x:c>
+      <x:c r="B4" s="85" t="str">
+        <x:v>Business or property researched for the requested market and customer profile.</x:v>
+      </x:c>
+      <x:c r="C4" s="85" t="str"/>
+      <x:c r="D4" s="85" t="str"/>
+      <x:c r="E4" s="85" t="str"/>
+      <x:c r="F4" s="85" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="85" t="str">
+        <x:v>Public contact path</x:v>
+      </x:c>
+      <x:c r="B5" s="85" t="str">
+        <x:v>Website, public business email, public phone, or other public business channel when available.</x:v>
+      </x:c>
+      <x:c r="C5" s="85" t="str"/>
+      <x:c r="D5" s="85" t="str"/>
+      <x:c r="E5" s="85" t="str"/>
+      <x:c r="F5" s="85" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="85" t="str">
+        <x:v>Why it fits</x:v>
+      </x:c>
+      <x:c r="B6" s="85" t="str">
+        <x:v>Short qualification note explaining why the prospect may match the buyer's offer.</x:v>
+      </x:c>
+      <x:c r="C6" s="85" t="str"/>
+      <x:c r="D6" s="85" t="str"/>
+      <x:c r="E6" s="85" t="str"/>
+      <x:c r="F6" s="85" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="85" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="B3" s="56" t="str">
-        <x:v>Meaning</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="20" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="B4" s="20" t="str">
-        <x:v>Start here: strongest fit / best first outreach</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="20" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="B5" s="20" t="str">
-        <x:v>Good fit: worth outreach after A-list</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="20" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="B6" s="20" t="str">
-        <x:v>Broader coverage: useful for scale and testing</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="42" customHeight="1">
-      <x:c r="A8" s="20" t="str">
-        <x:v>Names, contact details, and URLs in this sample are fictional. Real packs use public-source research and include source URLs.</x:v>
-      </x:c>
-      <x:c r="B8" s="20"/>
-      <x:c r="C8" s="20"/>
-      <x:c r="D8" s="20"/>
+      <x:c r="B7" s="85" t="str">
+        <x:v>A = start here, B = good fit, C = broader coverage.</x:v>
+      </x:c>
+      <x:c r="C7" s="85" t="str"/>
+      <x:c r="D7" s="85" t="str"/>
+      <x:c r="E7" s="85" t="str"/>
+      <x:c r="F7" s="85" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="85" t="str">
+        <x:v>Outreach angle</x:v>
+      </x:c>
+      <x:c r="B8" s="85" t="str">
+        <x:v>A prospect-specific reason or service fit for the first approach.</x:v>
+      </x:c>
+      <x:c r="C8" s="85" t="str"/>
+      <x:c r="D8" s="85" t="str"/>
+      <x:c r="E8" s="85" t="str"/>
+      <x:c r="F8" s="85" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="90" t="str">
+        <x:v>This sample is illustrative and uses fictional names/contact details. A real deliverable is researched for the client's actual service, geography, exclusions, and ideal customer. Public contact information is included only when it is available from public business sources.</x:v>
+      </x:c>
+      <x:c r="B10" s="90"/>
+      <x:c r="C10" s="90"/>
+      <x:c r="D10" s="90"/>
+      <x:c r="E10" s="90"/>
+      <x:c r="F10" s="90"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="90"/>
+      <x:c r="B11" s="90"/>
+      <x:c r="C11" s="90"/>
+      <x:c r="D11" s="90"/>
+      <x:c r="E11" s="90"/>
+      <x:c r="F11" s="90"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="90"/>
+      <x:c r="B12" s="90"/>
+      <x:c r="C12" s="90"/>
+      <x:c r="D12" s="90"/>
+      <x:c r="E12" s="90"/>
+      <x:c r="F12" s="90"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:D1"/>
-    <x:mergeCell ref="A8:D8"/>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A10:F12"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>